<commit_message>
Pipeline agents, ticket brief, medieval UI and reference updates
Requirement changes from Scout/Scribe now re-check Elf's scenarios, and
approved-scenario changes rebuild the TS workbook alongside dwarf:sync.
Also includes the QA pipeline, big room, ticket brief layout, automation
panel, overnight fixes, and new reference/ticket material.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scripts/eauto-insurance/output-results.xlsx
+++ b/scripts/eauto-insurance/output-results.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="29">
   <si>
     <t>Vehicle Number</t>
   </si>
@@ -50,26 +50,62 @@
     <t>Total Price</t>
   </si>
   <si>
+    <t>VPM7358</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PERODUA </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Perodua Myvi 1500 AV </t>
+  </si>
+  <si>
+    <t xml:space="preserve">2022 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1496 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 SP AUTOMATIC CONSTANTLY VARI </t>
+  </si>
+  <si>
+    <t xml:space="preserve">AV MY17 FACELIFT </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chubb </t>
+  </si>
+  <si>
+    <t>Cover Type Private Car (Enhanced)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No </t>
+  </si>
+  <si>
+    <t xml:space="preserve">[Sum Insured more than -8.51 % below market value is Decline Risk.] </t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lonpac </t>
+  </si>
+  <si>
+    <t>Cover Type Comprehensive (1st party)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vehicle class does not match the class code </t>
+  </si>
+  <si>
     <t>Status</t>
   </si>
   <si>
     <t>Reason</t>
-  </si>
-  <si>
-    <t>VPM7358</t>
-  </si>
-  <si>
-    <t>NO_VEHICLE_INFO</t>
-  </si>
-  <si>
-    <t>Unable to retrieve your vehicle information</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -80,6 +116,10 @@
     <font>
       <b/>
       <color rgb="FFFFFFFF"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFF0000"/>
     </font>
   </fonts>
   <fills count="4">
@@ -112,11 +152,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -457,7 +498,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -511,7 +552,84 @@
         <v>11</v>
       </c>
     </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H2" t="s">
+        <v>19</v>
+      </c>
+      <c r="I2" t="s">
+        <v>20</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="K2" t="s">
+        <v>22</v>
+      </c>
+      <c r="L2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" t="s">
+        <v>17</v>
+      </c>
+      <c r="G3" t="s">
+        <v>18</v>
+      </c>
+      <c r="H3" t="s">
+        <v>24</v>
+      </c>
+      <c r="I3" t="s">
+        <v>25</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="K3" t="s">
+        <v>26</v>
+      </c>
+      <c r="L3" t="s">
+        <v>23</v>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="A1:L3"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -519,7 +637,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -527,26 +645,15 @@
     <col min="3" max="3" width="60" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C2" t="s">
-        <v>16</v>
+      <c r="B1" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>